<commit_message>
Data. Reentrenamiento de modelos y nuevo assess para ITA y GER
</commit_message>
<xml_diff>
--- a/p6_deployment/data/england/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/p6_deployment/data/england/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1003,2230 +1003,2354 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>tYjCfe2E</t>
+          <t>fmqtFMjD</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45514.45833333334</v>
+        <v>45522.52083333334</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
+          <t xml:space="preserve">stamford bridge
+  london </t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>40341</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K10" t="n">
+        <v>481</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>AeRSxQrK</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45523.66666666666</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" t="n">
+        <v>481</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>tYjCfe2E</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45514.45833333334</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
           <t xml:space="preserve">wembley stadium
   london </t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E12" t="n">
         <v>90000</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>ppjDR086</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>manchester utd</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Wtn9Stg0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>manchester city</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>48</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
         <v>482</v>
       </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="n">
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
         <v>2024</v>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>fa community shield</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>OMDVg8x9</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
         <is>
           <t xml:space="preserve">brunton park
   carlisle </t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E13" t="n">
         <v>17949</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>dUzTIwSF</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>carlisle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>hSUajdSS</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>stoke</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>48</v>
-      </c>
-      <c r="K11" t="n">
-        <v>484</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>484</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>jXcAnQUr</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B14" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
         <is>
           <t xml:space="preserve">brisbane road
   london </t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E14" t="n">
         <v>9271</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>KKyYcus9</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>leyton orient</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>ChwgcrNJ</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>newport</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>48</v>
-      </c>
-      <c r="K12" t="n">
-        <v>484</v>
-      </c>
-      <c r="L12" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>484</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>fRe0c20b</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t xml:space="preserve">edgeley park
   stockport </t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E15" t="n">
         <v>10841</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>IX6WjNvr</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>stockport county</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>6Nl8nagD</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>blackburn</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>48</v>
-      </c>
-      <c r="K13" t="n">
-        <v>484</v>
-      </c>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>484</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>CnnJp4ae</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B16" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
         <is>
           <t xml:space="preserve">holker street
   barrow in furness </t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E16" t="n">
         <v>6500</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>KKJL7QXd</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>barrow</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>U3lM3y4e</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>port vale</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
-        <v>484</v>
-      </c>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>484</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>bw1zAKS6</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
         <is>
           <t xml:space="preserve">toughsheet community stadium
   bolton </t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E17" t="n">
         <v>28723</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Or1bBrWD</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>bolton</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>t6G9wMZN</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>mansfield</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
-        <v>484</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>484</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>GINCsvmn</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B18" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t xml:space="preserve">ashton gate stadium
   bristol </t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E18" t="n">
         <v>27000</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>MahqU27I</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>bristol city</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>GOvB22xg</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>coventry</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
-        <v>484</v>
-      </c>
-      <c r="L16" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>484</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>x6klsVh3</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B19" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
         <is>
           <t xml:space="preserve">hayes lane
   london </t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E19" t="n">
         <v>5000</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Opdcd08Q</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>bromley</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>4KREuF43</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>afc wimbledon</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
-        <v>484</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="J19" t="n">
+        <v>48</v>
+      </c>
+      <c r="K19" t="n">
+        <v>484</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>b3pRrrU7</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
         <is>
           <t xml:space="preserve">pirelli stadium
   burton upon trent </t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E20" t="n">
         <v>6912</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>nwCtJaJT</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>burton</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>8EFIJthC</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>blackpool</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>48</v>
-      </c>
-      <c r="K18" t="n">
-        <v>484</v>
-      </c>
-      <c r="L18" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="J20" t="n">
+        <v>48</v>
+      </c>
+      <c r="K20" t="n">
+        <v>484</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>WfkfPdXH</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B21" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
         <is>
           <t xml:space="preserve">abbey stadium
   cambridge </t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E21" t="n">
         <v>7937</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>lnb8EJRp</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>cambridge utd</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>lrMHUHDc</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>qpr</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>48</v>
-      </c>
-      <c r="K19" t="n">
-        <v>484</v>
-      </c>
-      <c r="L19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="J21" t="n">
+        <v>48</v>
+      </c>
+      <c r="K21" t="n">
+        <v>484</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>SMr3Nz2U</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
         <is>
           <t xml:space="preserve">cardiff city stadium
   cardiff </t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E22" t="n">
         <v>33280</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>hO8wh6aP</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>cardiff</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>GILi6JC9</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>bristol rovers</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>48</v>
-      </c>
-      <c r="K20" t="n">
-        <v>484</v>
-      </c>
-      <c r="L20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="J22" t="n">
+        <v>48</v>
+      </c>
+      <c r="K22" t="n">
+        <v>484</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>xYBLuIHb</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t xml:space="preserve">the valley
   london </t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E23" t="n">
         <v>27111</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>fXf5mQ7t</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>charlton</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>SWk4muv7</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>birmingham</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>48</v>
-      </c>
-      <c r="K21" t="n">
-        <v>484</v>
-      </c>
-      <c r="L21" t="n">
-        <v>1</v>
-      </c>
-      <c r="M21" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="J23" t="n">
+        <v>48</v>
+      </c>
+      <c r="K23" t="n">
+        <v>484</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>6os5wmhS</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B24" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t xml:space="preserve">colchester community stadium
   colchester </t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E24" t="n">
         <v>10105</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>xYu73rNn</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>colchester</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>EmlVDpVP</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>reading</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>48</v>
-      </c>
-      <c r="K22" t="n">
-        <v>484</v>
-      </c>
-      <c r="L22" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="J24" t="n">
+        <v>48</v>
+      </c>
+      <c r="K24" t="n">
+        <v>484</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>Kl7vhn7L</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B25" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">the broadfield stadium
   crawley </t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E25" t="n">
         <v>6134</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>QVmLl54o</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>crawley</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>xSloasB8</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>swindon</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>48</v>
-      </c>
-      <c r="K23" t="n">
-        <v>484</v>
-      </c>
-      <c r="L23" t="n">
-        <v>1</v>
-      </c>
-      <c r="M23" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="J25" t="n">
+        <v>48</v>
+      </c>
+      <c r="K25" t="n">
+        <v>484</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>nw6fJO5K</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B26" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
         <is>
           <t xml:space="preserve">pride park
   derby </t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="E26" t="n">
         <v>33597</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Iug0YO0Q</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>derby</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>dQIMIN5n</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>chesterfield</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>48</v>
-      </c>
-      <c r="K24" t="n">
-        <v>484</v>
-      </c>
-      <c r="L24" t="n">
-        <v>1</v>
-      </c>
-      <c r="M24" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="J26" t="n">
+        <v>48</v>
+      </c>
+      <c r="K26" t="n">
+        <v>484</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>bHPacsq1</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B27" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
         <is>
           <t xml:space="preserve">highbury stadium
   fleetwood </t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E27" t="n">
         <v>5327</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>tCZ3D68d</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>fleetwood</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>CCBWpzjj</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>west brom</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>48</v>
-      </c>
-      <c r="K25" t="n">
-        <v>484</v>
-      </c>
-      <c r="L25" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="J27" t="n">
+        <v>48</v>
+      </c>
+      <c r="K27" t="n">
+        <v>484</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>MwmHgKaN</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B28" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t xml:space="preserve">blundell park
   cleethorpes </t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E28" t="n">
         <v>9052</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>OEaiS3za</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>grimsby</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>bsc3EJ27</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>bradford city</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>48</v>
-      </c>
-      <c r="K26" t="n">
-        <v>484</v>
-      </c>
-      <c r="L26" t="n">
-        <v>1</v>
-      </c>
-      <c r="M26" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="J28" t="n">
+        <v>48</v>
+      </c>
+      <c r="K28" t="n">
+        <v>484</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>lQl9etVA</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">john smith s stadium
   huddersfield </t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E29" t="n">
         <v>24121</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>xxxpBZl2</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>huddersfield</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>zmKRcPKu</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>morecambe</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>48</v>
-      </c>
-      <c r="K27" t="n">
-        <v>484</v>
-      </c>
-      <c r="L27" t="n">
-        <v>1</v>
-      </c>
-      <c r="M27" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="J29" t="n">
+        <v>48</v>
+      </c>
+      <c r="K29" t="n">
+        <v>484</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>KWD8eLDD</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
         <is>
           <t xml:space="preserve">lner stadium
   lincoln </t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="E30" t="n">
         <v>10669</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>hrHTRs5B</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>lincoln</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>CQv5qrFt</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>harrogate</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>48</v>
-      </c>
-      <c r="K28" t="n">
-        <v>484</v>
-      </c>
-      <c r="L28" t="n">
-        <v>1</v>
-      </c>
-      <c r="M28" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="J30" t="n">
+        <v>48</v>
+      </c>
+      <c r="K30" t="n">
+        <v>484</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>xUXzYQFk</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t xml:space="preserve">sixfields stadium
   northampton </t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E31" t="n">
         <v>7798</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>l4P6dwRR</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>northampton</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>hl2V5JIl</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>wycombe</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>48</v>
-      </c>
-      <c r="K29" t="n">
-        <v>484</v>
-      </c>
-      <c r="L29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M29" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="J31" t="n">
+        <v>48</v>
+      </c>
+      <c r="K31" t="n">
+        <v>484</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>CCV9JR0d</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B32" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
         <is>
           <t xml:space="preserve">carrow road
   norwich </t>
         </is>
       </c>
-      <c r="E30" t="n">
+      <c r="E32" t="n">
         <v>27137</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Qo6off6p</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>norwich</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>ANwyQM2M</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>stevenage</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>48</v>
-      </c>
-      <c r="K30" t="n">
-        <v>484</v>
-      </c>
-      <c r="L30" t="n">
-        <v>1</v>
-      </c>
-      <c r="M30" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="J32" t="n">
+        <v>48</v>
+      </c>
+      <c r="K32" t="n">
+        <v>484</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1</v>
+      </c>
+      <c r="M32" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>bsinRI25</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B33" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
         <is>
           <t xml:space="preserve">kassam stadium
   oxford </t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E33" t="n">
         <v>12500</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>vgOBT43c</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>oxford utd</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>tWeI85kh</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>peterborough</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>48</v>
-      </c>
-      <c r="K31" t="n">
-        <v>484</v>
-      </c>
-      <c r="L31" t="n">
-        <v>1</v>
-      </c>
-      <c r="M31" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="J33" t="n">
+        <v>48</v>
+      </c>
+      <c r="K33" t="n">
+        <v>484</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>GbaVU03t</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B34" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">fratton park
   portsmouth </t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E34" t="n">
         <v>21944</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>zckREQFJ</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>portsmouth</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>6uz2cJBL</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>millwall</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>48</v>
-      </c>
-      <c r="K32" t="n">
-        <v>484</v>
-      </c>
-      <c r="L32" t="n">
-        <v>1</v>
-      </c>
-      <c r="M32" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="J34" t="n">
+        <v>48</v>
+      </c>
+      <c r="K34" t="n">
+        <v>484</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>tOTmlbNp</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">deepdale
   preston </t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E35" t="n">
         <v>23408</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>x8IDVcbi</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>preston</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>WSzc94ws</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>sunderland</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>48</v>
-      </c>
-      <c r="K33" t="n">
-        <v>484</v>
-      </c>
-      <c r="L33" t="n">
-        <v>1</v>
-      </c>
-      <c r="M33" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="J35" t="n">
+        <v>48</v>
+      </c>
+      <c r="K35" t="n">
+        <v>484</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>nPQL4PjR</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
         <is>
           <t xml:space="preserve">aesseal new york stadium
   rotherham </t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E36" t="n">
         <v>12021</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>KMfM7P4b</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>rotherham</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>YacqHHdS</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>crewe</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>48</v>
-      </c>
-      <c r="K34" t="n">
-        <v>484</v>
-      </c>
-      <c r="L34" t="n">
-        <v>1</v>
-      </c>
-      <c r="M34" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="J36" t="n">
+        <v>48</v>
+      </c>
+      <c r="K36" t="n">
+        <v>484</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>pWhdu9NF</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B37" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">peninsula stadium
   salford </t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E37" t="n">
         <v>5108</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>W4AadhN3</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>salford</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>hlzYDy5q</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>doncaster</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>48</v>
-      </c>
-      <c r="K35" t="n">
-        <v>484</v>
-      </c>
-      <c r="L35" t="n">
-        <v>1</v>
-      </c>
-      <c r="M35" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="J37" t="n">
+        <v>48</v>
+      </c>
+      <c r="K37" t="n">
+        <v>484</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>6NnRD2Ts</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B38" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
         <is>
           <t xml:space="preserve">the croud meadow
   shrewsbury </t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E38" t="n">
         <v>9877</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>EqfQ6qK4</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>shrewsbury</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>EwJVdqzn</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>notts co</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>48</v>
-      </c>
-      <c r="K36" t="n">
-        <v>484</v>
-      </c>
-      <c r="L36" t="n">
-        <v>1</v>
-      </c>
-      <c r="M36" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="J38" t="n">
+        <v>48</v>
+      </c>
+      <c r="K38" t="n">
+        <v>484</v>
+      </c>
+      <c r="L38" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>2FcwTvYh</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B39" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
         <is>
           <t xml:space="preserve">swansea com stadium
   swansea </t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E39" t="n">
         <v>21088</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>K6xezbY7</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>swansea</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>WvZyDeKk</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>gillingham</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>48</v>
-      </c>
-      <c r="K37" t="n">
-        <v>484</v>
-      </c>
-      <c r="L37" t="n">
-        <v>1</v>
-      </c>
-      <c r="M37" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="J39" t="n">
+        <v>48</v>
+      </c>
+      <c r="K39" t="n">
+        <v>484</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>EBSD6oME</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B40" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
         <is>
           <t xml:space="preserve">prenton park
   birkenhead </t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E40" t="n">
         <v>16587</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>jVhkb1QE</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>tranmere</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>6ZvdGuYf</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>accrington</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>48</v>
-      </c>
-      <c r="K38" t="n">
-        <v>484</v>
-      </c>
-      <c r="L38" t="n">
-        <v>1</v>
-      </c>
-      <c r="M38" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+      <c r="J40" t="n">
+        <v>48</v>
+      </c>
+      <c r="K40" t="n">
+        <v>484</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>WSQqW4p2</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B41" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
         <is>
           <t xml:space="preserve">bescot stadium
   walsall </t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E41" t="n">
         <v>11300</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>YgrfcLuL</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>walsall</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>ve14a3l4</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>exeter</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>48</v>
-      </c>
-      <c r="K39" t="n">
-        <v>484</v>
-      </c>
-      <c r="L39" t="n">
-        <v>1</v>
-      </c>
-      <c r="M39" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+      <c r="J41" t="n">
+        <v>48</v>
+      </c>
+      <c r="K41" t="n">
+        <v>484</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>vaX1LmWq</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B42" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
         <is>
           <t xml:space="preserve">vicarage road
   watford </t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E42" t="n">
         <v>22200</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>UmMRoGzp</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>watford</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>f9KDxtkU</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>mk dons</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>48</v>
-      </c>
-      <c r="K40" t="n">
-        <v>484</v>
-      </c>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+      <c r="J42" t="n">
+        <v>48</v>
+      </c>
+      <c r="K42" t="n">
+        <v>484</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>n1hhaOVo</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B43" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
         <is>
           <t xml:space="preserve">dw stadium
   wigan </t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E43" t="n">
         <v>25133</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>MgHlK2Na</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>wigan</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>UNGEKMx6</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>barnsley</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>48</v>
-      </c>
-      <c r="K41" t="n">
-        <v>484</v>
-      </c>
-      <c r="L41" t="n">
-        <v>1</v>
-      </c>
-      <c r="M41" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+      <c r="J43" t="n">
+        <v>48</v>
+      </c>
+      <c r="K43" t="n">
+        <v>484</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>vyoZBtbf</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>45517.66666666666</v>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
         <is>
           <t xml:space="preserve">bramall lane
   sheffield </t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E44" t="n">
         <v>32050</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>MeKPSerA</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>sheffield utd</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>IgO7K1ZA</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>wrexham</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>48</v>
-      </c>
-      <c r="K42" t="n">
-        <v>484</v>
-      </c>
-      <c r="L42" t="n">
-        <v>1</v>
-      </c>
-      <c r="M42" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+      <c r="J44" t="n">
+        <v>48</v>
+      </c>
+      <c r="K44" t="n">
+        <v>484</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>634r8bcJ</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B45" s="2" t="n">
         <v>45518.65625</v>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
         <is>
           <t xml:space="preserve">mkm stadium
   hull </t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E45" t="n">
         <v>25586</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>S66R0t75</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>hull</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>llcCvIcG</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>sheffield wed</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>48</v>
-      </c>
-      <c r="K43" t="n">
-        <v>484</v>
-      </c>
-      <c r="L43" t="n">
-        <v>1</v>
-      </c>
-      <c r="M43" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+      <c r="J45" t="n">
+        <v>48</v>
+      </c>
+      <c r="K45" t="n">
+        <v>484</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>pbFTwdnB</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B46" s="2" t="n">
         <v>45518.65625</v>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
         <is>
           <t xml:space="preserve">home park
   plymouth </t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E46" t="n">
         <v>17000</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>WpGM6ELj</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>plymouth</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>jizXHcsM</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>cheltenham</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>48</v>
-      </c>
-      <c r="K44" t="n">
-        <v>484</v>
-      </c>
-      <c r="L44" t="n">
-        <v>1</v>
-      </c>
-      <c r="M44" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+      <c r="J46" t="n">
+        <v>48</v>
+      </c>
+      <c r="K46" t="n">
+        <v>484</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1</v>
+      </c>
+      <c r="M46" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>efl cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>697ha3El</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B47" s="2" t="n">
         <v>45518.66666666666</v>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
         <is>
           <t xml:space="preserve">elland road
   leeds </t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E47" t="n">
         <v>37792</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>tUxUbLR2</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>leeds</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>6F0lvLNC</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>middlesbrough</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>48</v>
-      </c>
-      <c r="K45" t="n">
-        <v>484</v>
-      </c>
-      <c r="L45" t="n">
-        <v>1</v>
-      </c>
-      <c r="M45" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
+      <c r="J47" t="n">
+        <v>48</v>
+      </c>
+      <c r="K47" t="n">
+        <v>484</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>

</xml_diff>